<commit_message>
Initial commit: Stabilized LedgerFlow Agent pipeline, fixed Pydantic schemas, and configured memory.
</commit_message>
<xml_diff>
--- a/verified_data.xlsx
+++ b/verified_data.xlsx
@@ -476,245 +476,205 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Cost of Sales</t>
-        </is>
-      </c>
+          <t>2001.1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Cash Sale Debit</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>884.0</t>
+          <t>5000.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>214</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Trading account</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Cost of Sales</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
+          <t>2001.2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Cash Sale Credit</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>884.0</t>
+          <t>5000.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>125</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2002.1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Other Expenses</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Service Revenue Debit</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1120.0</t>
+          <t>7200.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>350</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Trading account</t>
+          <t>Operating account</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Operating Expenses</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
+          <t>2002.2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1120.0</t>
-        </is>
-      </c>
+          <t>Service Revenue Credit</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>7000.0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>328</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Advertisements</t>
-        </is>
-      </c>
+          <t>2003.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Credit Expenses</t>
+          <t>Inventory Purchase Debit</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2394.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>854</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -727,47 +687,35 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Operating account</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Operating Expenses</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Accrued Expenses</t>
-        </is>
-      </c>
+          <t>2003.2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Credit Expenses</t>
+          <t>Inventory Purchase Credit</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2394.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>204</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -780,259 +728,199 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Liabilities and Owners Equity</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Liabilities</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>2004.1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Credit Sales</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2948.0</t>
-        </is>
-      </c>
+          <t>Office Rent Debit</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3000.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>658</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Trading account</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4.2</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Trade Receivables</t>
-        </is>
-      </c>
+          <t>2004.2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Credit Sales</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2940.0</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Office Rent Credit</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2700.0</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>189</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>2005.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cash Sales</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>3734.0</t>
-        </is>
-      </c>
+          <t>Equipment Purchase Debit</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>15000.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>532</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Trading account</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>5.2</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Cash at Bank</t>
-        </is>
-      </c>
+          <t>2005.2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cash Sales</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>3723.0</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Equipment Purchase Credit</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>15000.0</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>132</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Cost of Sales</t>
-        </is>
-      </c>
+          <t>2006.1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Salary Expense Debit</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4371.0</t>
+          <t>8500.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>195</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1045,47 +933,35 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Trading account</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Cost of Sales</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
+          <t>2006.2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cost of Sales</t>
+          <t>Salary Expense Credit</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4371.0</t>
+          <t>8500.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>323</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1098,47 +974,35 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>2007.1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Credit Sales</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>14570.0</t>
-        </is>
-      </c>
+          <t>Insurance Payment Debit</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>716</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1151,47 +1015,35 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Trading account</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2018-01-01 00:00:00</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Trade Receivables</t>
-        </is>
-      </c>
+          <t>2007.2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Credit Sales</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>14570.0</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>Insurance Payment Credit</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>3700.0</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>127</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1204,16 +1056,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Assets</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>